<commit_message>
Last Phase m — another maintainer’s manual review
</commit_message>
<xml_diff>
--- a/dev/review_manual/Excel_stars.xlsx
+++ b/dev/review_manual/Excel_stars.xlsx
@@ -1040,17 +1040,17 @@
       </c>
       <c r="C3" s="49" t="inlineStr">
         <is>
-          <t>1-Democrat</t>
+          <t>Democrat</t>
         </is>
       </c>
       <c r="D3" s="48" t="inlineStr">
         <is>
-          <t>2-Independent, other</t>
+          <t>Independent, other</t>
         </is>
       </c>
       <c r="E3" s="48" t="inlineStr">
         <is>
-          <t>3-Republican</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="F3" s="49" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="B8" s="58" t="inlineStr">
         <is>
-          <t>1-Lt $10000</t>
+          <t>Lt $10000</t>
         </is>
       </c>
       <c r="C8" s="113">
@@ -1291,7 +1291,7 @@
       <c r="A9" s="53"/>
       <c r="B9" s="52" t="inlineStr">
         <is>
-          <t>2-$10000 to 14999</t>
+          <t>$10000 to 14999</t>
         </is>
       </c>
       <c r="C9" s="114">
@@ -1329,7 +1329,7 @@
       <c r="A10" s="53"/>
       <c r="B10" s="52" t="inlineStr">
         <is>
-          <t>3-$15000 to 24999</t>
+          <t>$15000 to 24999</t>
         </is>
       </c>
       <c r="C10" s="114">
@@ -1367,7 +1367,7 @@
       <c r="A11" s="53"/>
       <c r="B11" s="52" t="inlineStr">
         <is>
-          <t>4-$25000 or more</t>
+          <t>$25000 or more</t>
         </is>
       </c>
       <c r="C11" s="114">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="B13" s="58" t="inlineStr">
         <is>
-          <t>1-Protestant</t>
+          <t>Protestant</t>
         </is>
       </c>
       <c r="C13" s="113">
@@ -1485,7 +1485,7 @@
       <c r="A14" s="53"/>
       <c r="B14" s="52" t="inlineStr">
         <is>
-          <t>2-Catholic</t>
+          <t>Catholic</t>
         </is>
       </c>
       <c r="C14" s="73">
@@ -1523,7 +1523,7 @@
       <c r="A15" s="53"/>
       <c r="B15" s="52" t="inlineStr">
         <is>
-          <t>3-Other christian</t>
+          <t>Other christian</t>
         </is>
       </c>
       <c r="C15" s="114">
@@ -1561,7 +1561,7 @@
       <c r="A16" s="53"/>
       <c r="B16" s="52" t="inlineStr">
         <is>
-          <t>4-Jewish</t>
+          <t>Jewish</t>
         </is>
       </c>
       <c r="C16" s="74">
@@ -1599,7 +1599,7 @@
       <c r="A17" s="53"/>
       <c r="B17" s="52" t="inlineStr">
         <is>
-          <t>5-Buddhist/Hinduist</t>
+          <t>Buddhist/Hinduist</t>
         </is>
       </c>
       <c r="C17" s="75">
@@ -1637,7 +1637,7 @@
       <c r="A18" s="53"/>
       <c r="B18" s="52" t="inlineStr">
         <is>
-          <t>6-Muslim</t>
+          <t>Muslim</t>
         </is>
       </c>
       <c r="C18" s="74">
@@ -1675,7 +1675,7 @@
       <c r="A19" s="53"/>
       <c r="B19" s="52" t="inlineStr">
         <is>
-          <t>7-Other</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C19" s="110">
@@ -1713,7 +1713,7 @@
       <c r="A20" s="53"/>
       <c r="B20" s="52" t="inlineStr">
         <is>
-          <t>8-None</t>
+          <t>None</t>
         </is>
       </c>
       <c r="C20" s="71">
@@ -1960,7 +1960,6 @@
           </r>
           <r>
             <rPr>
-              <b/>
               <sz val="9"/>
               <color rgb="FF6492B0"/>
               <rFont val="DejaVu Sans Condensed"/>
@@ -1976,7 +1975,6 @@
           </r>
           <r>
             <rPr>
-              <b/>
               <sz val="9"/>
               <color rgb="FF5E85B8"/>
               <rFont val="DejaVu Sans Condensed"/>
@@ -1992,7 +1990,6 @@
           </r>
           <r>
             <rPr>
-              <b/>
               <sz val="9"/>
               <color rgb="FF5169C7"/>
               <rFont val="DejaVu Sans Condensed"/>
@@ -2022,7 +2019,6 @@
           </r>
           <r>
             <rPr>
-              <b/>
               <sz val="9"/>
               <color rgb="FFAE815E"/>
               <rFont val="DejaVu Sans Condensed"/>
@@ -2038,7 +2034,6 @@
           </r>
           <r>
             <rPr>
-              <b/>
               <sz val="9"/>
               <color rgb="FFB56E53"/>
               <rFont val="DejaVu Sans Condensed"/>
@@ -2054,7 +2049,6 @@
           </r>
           <r>
             <rPr>
-              <b/>
               <sz val="9"/>
               <color rgb="FFBE4034"/>
               <rFont val="DejaVu Sans Condensed"/>

</xml_diff>